<commit_message>
fix: repair expense upload template xlsx package
</commit_message>
<xml_diff>
--- a/templates/expense-upload.xlsx
+++ b/templates/expense-upload.xlsx
@@ -13,22 +13,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Member</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>

<commit_message>
chore: reorder expense template columns to match time flow
</commit_message>
<xml_diff>
--- a/templates/expense-upload.xlsx
+++ b/templates/expense-upload.xlsx
@@ -18,22 +18,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">

</xml_diff>